<commit_message>
Import real QuickBooks trial balance, aging, inventory and Journal exports
Recipes built on real QuickBooks Online exports (tests/fixtures/quickbooks/
kestrel_qbo/): trial balance, A/R aging summary, inventory valuation summary,
Journal (default and with Created on/by). A builder joins this year's and
last year's Trial Balance exports (API route and Sources panel). Kestrel's
files regenerated in the real layouts and loaded raw by the demo seed;
figures identical to the old hand-prepared loads, answer keys unchanged.

Fixed on the real files: abbreviated and whole-month period lines read as
undated; coverage counts a trial balance's line from the line mapping, only
when the mapping reaches a loaded account (review M1).

519 tests pass; finish-line 162/164, 0 unexplained; Oceanview unchanged.
Open: review M2, M3 and Lows; reconciliation import needs a PDF.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/case-studies/kestrel-valley-cycle/data/quickbooks/AR_Aging_Summary.xlsx
+++ b/case-studies/kestrel-valley-cycle/data/quickbooks/AR_Aging_Summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,22 +429,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A/R Aging Summary</t>
+          <t>A/R Aging Summary Report</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>As of June 30, 2026</t>
+          <t>As of Jun 30, 2026</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -464,7 +465,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>91 and over</t>
+          <t>91 AND OVER</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>